<commit_message>
import employee code template
</commit_message>
<xml_diff>
--- a/public/assets/import-templates/import-employees-template.xlsx
+++ b/public/assets/import-templates/import-employees-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\attendnace-project\3p-attend-front\public\assets\import-templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B53085D3-1CD8-45F5-ADA7-7CD182C16CD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8573BA46-38F0-4D06-BD24-E7F0DA47F80A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
     <t>JoinDate (mm/dd/yyyy)</t>
   </si>
   <si>
-    <t>EmployeeCode</t>
+    <t>EmployeeCode (xxxxxx)</t>
   </si>
 </sst>
 </file>
@@ -433,7 +433,7 @@
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="3" width="13.5703125" customWidth="1"/>
     <col min="4" max="4" width="12.85546875" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="22.7109375" style="3" customWidth="1"/>
     <col min="6" max="6" width="14.140625" style="3" customWidth="1"/>
     <col min="7" max="7" width="12.42578125" customWidth="1"/>
     <col min="8" max="8" width="9.7109375" customWidth="1"/>

</xml_diff>